<commit_message>
finished updating all to include all summer work (all work before the 9/25 SRKW quarterly meeting)
</commit_message>
<xml_diff>
--- a/Deliverables/ALL/MINOR-species-assignment-checks.xlsx
+++ b/Deliverables/ALL/MINOR-species-assignment-checks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid-my.sharepoint.com/personal/mball3_uw_edu/Documents/Documents/WADE LAB/SRKW/Deliverables/ALL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_6D63FDCE8F79A8D366075C52F3185237079EA177" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4332B9A4-1C9F-42C7-8785-D680812CA033}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_6D63FDCE8F79A8D366075C52F3185237079EA177" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{319E0BF1-0D36-4883-9E19-76B969A63FC3}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="698" yWindow="1163" windowWidth="19822" windowHeight="12517" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>species</t>
   </si>
@@ -170,6 +170,12 @@
   </si>
   <si>
     <t>Alaska pollock</t>
+  </si>
+  <si>
+    <t>100% in 1 Lysate sample</t>
+  </si>
+  <si>
+    <t>99% in 1 Lysate sample</t>
   </si>
 </sst>
 </file>
@@ -698,6 +704,9 @@
       <c r="C14" t="s">
         <v>27</v>
       </c>
+      <c r="D14" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
@@ -741,6 +750,9 @@
       </c>
       <c r="C18" t="s">
         <v>34</v>
+      </c>
+      <c r="D18" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.45">

</xml_diff>